<commit_message>
feat: pestaña Carros (gasolina) + fetch resiliente a tabs faltantes
- Nueva hoja 'Carros' en Gastos_Covenas.xlsx: ruta, presupuesto por carro
  (gasolina + peajes ida/vuelta), checklist, fuentes — mismo estilo que
  la hoja 'Tesla'.
- Lambda: separa rangos requeridos (Cabaña/Personas/Abonos/Gastos, en un
  solo batchGet, deben existir) de opcionales (Estimado/Tesla/Carros,
  pedidos uno por uno). Un tab opcional que no exista todavía en el
  Sheets real ya no tumba el dashboard entero con un 400 — degrada a
  grid vacío solo para esa pestaña.
- Frontend: pestaña 'Carros' reutilizando renderFreeformGrid, con mensaje
  claro cuando la pestaña aún no se ha copiado al Sheets compartido.

Nota: el .xlsx local ya no es la fuente viva (el Sheets real diverge desde
que se convirtió) — la pestaña 'Carros' vive en el archivo local hasta que
se copie manualmente al Sheets compartido (ver mensaje al usuario).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gastos_Covenas.xlsx
+++ b/Gastos_Covenas.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimado" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tesla" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carros" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4034,4 +4035,352 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>⛽ CARROS A GASOLINA — Medellín → Coveñas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="20" t="inlineStr">
+        <is>
+          <t>Ruta, presupuesto y checklist para los 2 carros a gasolina del grupo. Mismos supuestos que la hoja 'Estimado' — investigado en foros de peajes y guías de viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>RUTA Y PARADAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Km aprox. desde Medellín</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Qué hacer ahí</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>0 km</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>Salida</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>Tanquear lleno antes de salir — evita buscar bomba con poco tiempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Santa Fe de Antioquia / Caucasia</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>≈ 250 km</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Descanso + gasolina</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>Punto medio natural, hay estaciones de servicio y sitios para comer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>Planeta Rica / Sincelejo</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>≈ 350–400 km</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>Gasolina si hace falta</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>Segunda opción de tanqueo si no se llenó completo en Caucasia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>Coveñas / Tolú</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>≈ 500 km (destino)</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>Llegada</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>Confirmar parqueadero disponible en el condominio para los 2 carros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>PRESUPUESTO POR CARRO (ida y vuelta)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>Cálculo</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Estimado</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Fuente / nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>Gasolina (ida y vuelta)</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>≈500km ida x2 / 35 km-galón x $17.000/galón</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="n">
+        <v>486000</v>
+      </c>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>colombiapeajes.com / tarifas.info — rango real $340k-420k según rendimiento del carro</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>Peajes (ida y vuelta)</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>≈$80.000 por trayecto x2</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="n">
+        <v>160000</v>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>colombiapeajes.com — ruta Medellín-Coveñas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Total estimado por carro (ida y vuelta):</t>
+        </is>
+      </c>
+      <c r="C15" s="28">
+        <f>SUM(C13:C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Total 2 carros a gasolina:</t>
+        </is>
+      </c>
+      <c r="C16" s="28">
+        <f>C15*2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>CHECKLIST ANTES DE SALIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>☐  Revisión preventiva: llantas (incluida la de repuesto), frenos, aceite, luces, batería.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>☐  SOAT y tecnomecánica vigentes para la fecha del viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>☐  Kit de carretera: gato, cruceta, triángulos, chaleco reflectivo, botiquín, extintor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>☐  Tanquear lleno en Medellín antes de salir — no todas las paradas intermedias tienen bomba confiable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
+          <t>☐  Coordinar con el otro carro un punto de encuentro fijo si se separan en el camino.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="32" t="inlineStr">
+        <is>
+          <t>☐  Llevar efectivo para peajes (algunos puntos de la ruta no tienen pago electrónico).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>☐  Descansar cada 2-3 horas de manejo — son cerca de 9 horas de carretera.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>☐  Guardar el recibo/soporte de gasolina y peajes si se va a repartir el gasto entre el carro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>FUENTES CONSULTADAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="34" t="inlineStr">
+        <is>
+          <t>—  colombiapeajes.com — peajes ruta Medellín-Coveñas</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="34" t="inlineStr">
+        <is>
+          <t>—  tarifas.info — gasolina y peajes Medellín-Coveñas 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="34" t="inlineStr">
+        <is>
+          <t>—  yotellevo.net / himmera.com — distancia y tiempo de viaje Medellín-Coveñas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>